<commit_message>
Fit PC4's lifetime from 1500 ns, as the published value was
PC4's decay has a fast early component ahead of the triplet, and the
automatic fit start (about 500 ns after the pulse) folds both into one
exponential, giving 1228.49 ns. The published 1494.54 ns came from the same
fit opened at a fixed 1500 ns on the instrument time axis. FIT_START_NS
in lifetimes_tcspc.py now does that for PC4 only, and reproduces the
original re-fits to every printed digit (1494.54 +/- 19.32 ns; the repeat
gives 1381.92). All 27 screened lifetimes now match the curated table, and
no other photocatalyst changes.

PC4's k_q and k_q floor scale by 0.822 across its 48 pairs; K_SV and
every label are unchanged. Benchmark MCCs move by at most 0.003 (0.010
for one leave-one-PC-out entry), none of them a quoted number.
</commit_message>
<xml_diff>
--- a/data/experimental_data_processed/photocatalyst_properties_exp.xlsx
+++ b/data/experimental_data_processed/photocatalyst_properties_exp.xlsx
@@ -767,13 +767,13 @@
         <v>490</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>1228.49</v>
+        <v>1494.54</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>133.891</v>
+        <v>79.6344</v>
       </c>
       <c r="K6" s="10" t="n">
-        <v>0.108988</v>
+        <v>0.0532835</v>
       </c>
       <c r="L6" s="10" t="n">
         <v>2</v>
@@ -782,7 +782,7 @@
         <v>2</v>
       </c>
       <c r="N6" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6" s="10" t="inlineStr">
         <is>
@@ -791,7 +791,7 @@
       </c>
       <c r="P6" s="10" t="inlineStr">
         <is>
-          <t>longest of 2 measurements; measurements scatter by 11%, above the 10% threshold — needs a decision, not a rule; rejected 4_ACN_Ar_200ns_-5M_3mL_IrdFppy: window spans 3.6 lifetimes, below the 5 required; rejected 4_ACN_Ar_20us_-5M_3mL_IrdFppy: duplicate of 4_ACN_Ar_10us_-5M_3mL_IrdFppy</t>
+          <t>longest of 2 measurements; rejected 4_ACN_Ar_200ns_-5M_3mL_IrdFppy: not fitted; rejected 4_ACN_Ar_20us_-5M_3mL_IrdFppy: duplicate of 4_ACN_Ar_10us_-5M_3mL_IrdFppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Keep one lifetime trace per photocatalyst, named PC<n>
The TCSPC folder now holds exactly one trace per photocatalyst, as PC<n>.txt
and PC<n>.FL: the one behind each published lifetime. The alternative
traces, the second copies and PC7's lifetime are gone from the repository;
the originals stay in the parent project tree.

tau0 and its error are that trace's single-exponential fit and its
standard error, so lifetimes_tau0.py and its selection step are removed and
lifetimes_tcspc.py writes one row per photocatalyst. All 27 lifetimes and
their errors reproduce the published sheet to its two printed decimals.

pairs.csv carries tau0_err in place of tau0_rsd and tau0_consistent; no
lifetime, rate or benchmark result changes.
</commit_message>
<xml_diff>
--- a/data/experimental_data_processed/photocatalyst_properties_exp.xlsx
+++ b/data/experimental_data_processed/photocatalyst_properties_exp.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -485,12 +485,7 @@
     <col width="2" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="19" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
-    <col width="36" customWidth="1" min="15" max="15"/>
-    <col width="45" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
@@ -515,11 +510,6 @@
       </c>
       <c r="J1" s="6" t="n"/>
       <c r="K1" s="6" t="n"/>
-      <c r="L1" s="6" t="n"/>
-      <c r="M1" s="6" t="n"/>
-      <c r="N1" s="6" t="n"/>
-      <c r="O1" s="6" t="n"/>
-      <c r="P1" s="6" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
@@ -559,35 +549,10 @@
       </c>
       <c r="J2" s="9" t="inlineStr">
         <is>
-          <t>tau0_std / ns</t>
+          <t>tau0_err / ns</t>
         </is>
       </c>
       <c r="K2" s="9" t="inlineStr">
-        <is>
-          <t>tau0_rsd</t>
-        </is>
-      </c>
-      <c r="L2" s="9" t="inlineStr">
-        <is>
-          <t>n_measurements</t>
-        </is>
-      </c>
-      <c r="M2" s="9" t="inlineStr">
-        <is>
-          <t>n_traces_rejected</t>
-        </is>
-      </c>
-      <c r="N2" s="9" t="inlineStr">
-        <is>
-          <t>tau0_consistent</t>
-        </is>
-      </c>
-      <c r="O2" s="9" t="inlineStr">
-        <is>
-          <t>trace_used</t>
-        </is>
-      </c>
-      <c r="P2" s="9" t="inlineStr">
         <is>
           <t>tau0_note</t>
         </is>
@@ -622,26 +587,7 @@
       <c r="J3" s="10" t="n">
         <v>5.30814</v>
       </c>
-      <c r="K3" s="10" t="n">
-        <v>0.00222302</v>
-      </c>
-      <c r="L3" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M3" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="10" t="n"/>
-      <c r="O3" s="10" t="inlineStr">
-        <is>
-          <t>1_ACN_Ar_20us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P3" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="10" t="n">
@@ -672,26 +618,7 @@
       <c r="J4" s="10" t="n">
         <v>1.70003</v>
       </c>
-      <c r="K4" s="10" t="n">
-        <v>0.00305149</v>
-      </c>
-      <c r="L4" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M4" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="10" t="n"/>
-      <c r="O4" s="10" t="inlineStr">
-        <is>
-          <t>2_ACN_Ar_10us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P4" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="10" t="n">
@@ -722,26 +649,7 @@
       <c r="J5" s="10" t="n">
         <v>4.13219</v>
       </c>
-      <c r="K5" s="10" t="n">
-        <v>0.00243308</v>
-      </c>
-      <c r="L5" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M5" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" s="10" t="n"/>
-      <c r="O5" s="10" t="inlineStr">
-        <is>
-          <t>3_ACN_Ar_10us_-5M_3mL_Irppy</t>
-        </is>
-      </c>
-      <c r="P5" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error; rejected 3_ACN_Ar_20us_-5M_3mL_Irppy: duplicate of 3_ACN_Ar_10us_-5M_3mL_Irppy</t>
-        </is>
-      </c>
+      <c r="K5" s="10" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="10" t="n">
@@ -770,28 +678,11 @@
         <v>1494.54</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>79.6344</v>
-      </c>
-      <c r="K6" s="10" t="n">
-        <v>0.0532835</v>
-      </c>
-      <c r="L6" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="M6" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="N6" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="O6" s="10" t="inlineStr">
-        <is>
-          <t>4_ACN_Ar_10us_-5M_3mL_IrdFppy</t>
-        </is>
-      </c>
-      <c r="P6" s="10" t="inlineStr">
-        <is>
-          <t>longest of 2 measurements; rejected 4_ACN_Ar_200ns_-5M_3mL_IrdFppy: not fitted; rejected 4_ACN_Ar_20us_-5M_3mL_IrdFppy: duplicate of 4_ACN_Ar_10us_-5M_3mL_IrdFppy</t>
+        <v>19.3165</v>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>fit start fixed at 1500 ns</t>
         </is>
       </c>
     </row>
@@ -824,26 +715,7 @@
       <c r="J7" s="10" t="n">
         <v>2.1878</v>
       </c>
-      <c r="K7" s="10" t="n">
-        <v>0.00250407</v>
-      </c>
-      <c r="L7" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="10" t="n"/>
-      <c r="O7" s="10" t="inlineStr">
-        <is>
-          <t>5_ACN_Ar_10us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P7" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="n">
@@ -874,26 +746,7 @@
       <c r="J8" s="10" t="n">
         <v>1.82806</v>
       </c>
-      <c r="K8" s="10" t="n">
-        <v>0.00291845</v>
-      </c>
-      <c r="L8" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="10" t="n"/>
-      <c r="O8" s="10" t="inlineStr">
-        <is>
-          <t>6_ACN_Ar_10us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P8" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K8" s="10" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="n">
@@ -914,32 +767,9 @@
       </c>
       <c r="F9" s="10" t="n"/>
       <c r="G9" s="10" t="n"/>
-      <c r="I9" s="10" t="n">
-        <v>0.255827</v>
-      </c>
-      <c r="J9" s="10" t="n">
-        <v>0.00118839</v>
-      </c>
-      <c r="K9" s="10" t="n">
-        <v>0.00464529</v>
-      </c>
-      <c r="L9" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M9" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="10" t="n"/>
-      <c r="O9" s="10" t="inlineStr">
-        <is>
-          <t>7_ACN_Ar_10ns_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P9" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="I9" s="10" t="n"/>
+      <c r="J9" s="10" t="n"/>
+      <c r="K9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="n">
@@ -970,26 +800,7 @@
       <c r="J10" s="10" t="n">
         <v>14.9412</v>
       </c>
-      <c r="K10" s="10" t="n">
-        <v>0.00232049</v>
-      </c>
-      <c r="L10" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M10" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="10" t="n"/>
-      <c r="O10" s="10" t="inlineStr">
-        <is>
-          <t>8_ACN_Ar_50us_-5M_3mL_IrCF3pmb</t>
-        </is>
-      </c>
-      <c r="P10" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="n">
@@ -1020,26 +831,7 @@
       <c r="J11" s="10" t="n">
         <v>4.73231</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>0.00204433</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="10" t="n"/>
-      <c r="O11" s="10" t="inlineStr">
-        <is>
-          <t>9_ACN_Ar_20us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P11" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="n">
@@ -1070,26 +862,7 @@
       <c r="J12" s="10" t="n">
         <v>0.206387</v>
       </c>
-      <c r="K12" s="10" t="n">
-        <v>0.00276451</v>
-      </c>
-      <c r="L12" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="10" t="n"/>
-      <c r="O12" s="10" t="inlineStr">
-        <is>
-          <t>10_ACN_Ar_1us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P12" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="n">
@@ -1120,26 +893,7 @@
       <c r="J13" s="10" t="n">
         <v>3.82431</v>
       </c>
-      <c r="K13" s="10" t="n">
-        <v>0.00287235</v>
-      </c>
-      <c r="L13" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="10" t="n"/>
-      <c r="O13" s="10" t="inlineStr">
-        <is>
-          <t>11_ACN_Ar_20us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P13" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="n">
@@ -1170,26 +924,7 @@
       <c r="J14" s="10" t="n">
         <v>3.903</v>
       </c>
-      <c r="K14" s="10" t="n">
-        <v>0.0027297</v>
-      </c>
-      <c r="L14" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M14" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="10" t="n"/>
-      <c r="O14" s="10" t="inlineStr">
-        <is>
-          <t>12_ACN_Ar_20us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P14" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="n">
@@ -1220,26 +955,7 @@
       <c r="J15" s="10" t="n">
         <v>5.07795</v>
       </c>
-      <c r="K15" s="10" t="n">
-        <v>0.0021741</v>
-      </c>
-      <c r="L15" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M15" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="10" t="n"/>
-      <c r="O15" s="10" t="inlineStr">
-        <is>
-          <t>13_ACN_Ar_20us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P15" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n">
@@ -1270,26 +986,7 @@
       <c r="J16" s="10" t="n">
         <v>4.93813</v>
       </c>
-      <c r="K16" s="10" t="n">
-        <v>0.00211888</v>
-      </c>
-      <c r="L16" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="10" t="n"/>
-      <c r="O16" s="10" t="inlineStr">
-        <is>
-          <t>14_ACN_Ar_20us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P16" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="n">
@@ -1318,30 +1015,9 @@
         <v>3417.56</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>119.027</v>
-      </c>
-      <c r="K17" s="10" t="n">
-        <v>0.0348281</v>
-      </c>
-      <c r="L17" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="M17" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="O17" s="10" t="inlineStr">
-        <is>
-          <t>15_ACN_Ar_50us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P17" s="10" t="inlineStr">
-        <is>
-          <t>longest of 2 measurements</t>
-        </is>
-      </c>
+        <v>9.249000000000001</v>
+      </c>
+      <c r="K17" s="10" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n">
@@ -1372,26 +1048,7 @@
       <c r="J18" s="10" t="n">
         <v>4.11826</v>
       </c>
-      <c r="K18" s="10" t="n">
-        <v>0.00267426</v>
-      </c>
-      <c r="L18" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="10" t="n"/>
-      <c r="O18" s="10" t="inlineStr">
-        <is>
-          <t>16_ACN_Ar_20us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P18" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="n">
@@ -1422,26 +1079,7 @@
       <c r="J19" s="10" t="n">
         <v>0.916385</v>
       </c>
-      <c r="K19" s="10" t="n">
-        <v>0.00330365</v>
-      </c>
-      <c r="L19" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="10" t="n"/>
-      <c r="O19" s="10" t="inlineStr">
-        <is>
-          <t>17_ACN_Ar_5us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P19" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K19" s="10" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n">
@@ -1472,26 +1110,7 @@
       <c r="J20" s="10" t="n">
         <v>9.456340000000001</v>
       </c>
-      <c r="K20" s="10" t="n">
-        <v>0.00258048</v>
-      </c>
-      <c r="L20" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="10" t="n"/>
-      <c r="O20" s="10" t="inlineStr">
-        <is>
-          <t>18_ACN_Ar_50us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P20" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="n">
@@ -1522,26 +1141,7 @@
       <c r="J21" s="10" t="n">
         <v>13.4651</v>
       </c>
-      <c r="K21" s="10" t="n">
-        <v>0.00283127</v>
-      </c>
-      <c r="L21" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" s="10" t="n"/>
-      <c r="O21" s="10" t="inlineStr">
-        <is>
-          <t>19_ACN_Ar_50us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P21" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K21" s="10" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n">
@@ -1572,26 +1172,7 @@
       <c r="J22" s="10" t="n">
         <v>4.09436</v>
       </c>
-      <c r="K22" s="10" t="n">
-        <v>0.00269511</v>
-      </c>
-      <c r="L22" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M22" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="10" t="n"/>
-      <c r="O22" s="10" t="inlineStr">
-        <is>
-          <t>20_ACN_Ar_20us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P22" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n">
@@ -1622,26 +1203,7 @@
       <c r="J23" s="10" t="n">
         <v>4.45561</v>
       </c>
-      <c r="K23" s="10" t="n">
-        <v>0.00222854</v>
-      </c>
-      <c r="L23" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" s="10" t="n"/>
-      <c r="O23" s="10" t="inlineStr">
-        <is>
-          <t>21_ACN_Ar_20us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P23" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n">
@@ -1670,30 +1232,9 @@
         <v>3304.66</v>
       </c>
       <c r="J24" s="10" t="n">
-        <v>111.136</v>
-      </c>
-      <c r="K24" s="10" t="n">
-        <v>0.03363</v>
-      </c>
-      <c r="L24" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="M24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="O24" s="10" t="inlineStr">
-        <is>
-          <t>22_ACN_Ar_50us_-5M_3mL_betterDegas</t>
-        </is>
-      </c>
-      <c r="P24" s="10" t="inlineStr">
-        <is>
-          <t>longest of 3 measurements</t>
-        </is>
-      </c>
+        <v>9.446070000000001</v>
+      </c>
+      <c r="K24" s="10" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="n">
@@ -1724,26 +1265,7 @@
       <c r="J25" s="10" t="n">
         <v>10.683</v>
       </c>
-      <c r="K25" s="10" t="n">
-        <v>0.00238048</v>
-      </c>
-      <c r="L25" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M25" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" s="10" t="n"/>
-      <c r="O25" s="10" t="inlineStr">
-        <is>
-          <t>23_ACN_Ar_50us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P25" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K25" s="10" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n">
@@ -1774,26 +1296,7 @@
       <c r="J26" s="10" t="n">
         <v>7.49855</v>
       </c>
-      <c r="K26" s="10" t="n">
-        <v>0.00561984</v>
-      </c>
-      <c r="L26" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M26" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="N26" s="10" t="n"/>
-      <c r="O26" s="10" t="inlineStr">
-        <is>
-          <t>24_ACN_Ar_10us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P26" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error; rejected 24_ACN_Ar_10ns_-5M_3mL: not fitted</t>
-        </is>
-      </c>
+      <c r="K26" s="10" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="n">
@@ -1824,26 +1327,7 @@
       <c r="J27" s="10" t="n">
         <v>3.76114</v>
       </c>
-      <c r="K27" s="10" t="n">
-        <v>0.00286086</v>
-      </c>
-      <c r="L27" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M27" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" s="10" t="n"/>
-      <c r="O27" s="10" t="inlineStr">
-        <is>
-          <t>25_ACN_Ar_20us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P27" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K27" s="10" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n">
@@ -1863,11 +1347,6 @@
       <c r="I28" s="10" t="n"/>
       <c r="J28" s="10" t="n"/>
       <c r="K28" s="10" t="n"/>
-      <c r="L28" s="10" t="n"/>
-      <c r="M28" s="10" t="n"/>
-      <c r="N28" s="10" t="n"/>
-      <c r="O28" s="10" t="n"/>
-      <c r="P28" s="10" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="n">
@@ -1898,26 +1377,7 @@
       <c r="J29" s="10" t="n">
         <v>2.06671</v>
       </c>
-      <c r="K29" s="10" t="n">
-        <v>0.00270585</v>
-      </c>
-      <c r="L29" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M29" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" s="10" t="n"/>
-      <c r="O29" s="10" t="inlineStr">
-        <is>
-          <t>27_ACN_Ar_10us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P29" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n">
@@ -1948,26 +1408,7 @@
       <c r="J30" s="10" t="n">
         <v>8.609540000000001</v>
       </c>
-      <c r="K30" s="10" t="n">
-        <v>0.00315807</v>
-      </c>
-      <c r="L30" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M30" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" s="10" t="n"/>
-      <c r="O30" s="10" t="inlineStr">
-        <is>
-          <t>28_ACN_Ar_50us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P30" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="n">
@@ -1998,32 +1439,13 @@
       <c r="J31" s="10" t="n">
         <v>4.24662</v>
       </c>
-      <c r="K31" s="10" t="n">
-        <v>0.00262042</v>
-      </c>
-      <c r="L31" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M31" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" s="10" t="n"/>
-      <c r="O31" s="10" t="inlineStr">
-        <is>
-          <t>29_ACN_Ar_20us_-5M_3mL</t>
-        </is>
-      </c>
-      <c r="P31" s="10" t="inlineStr">
-        <is>
-          <t>single measurement, within-fit standard error</t>
-        </is>
-      </c>
+      <c r="K31" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="I1:P1"/>
     <mergeCell ref="E1:G1"/>
+    <mergeCell ref="I1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2035,7 +1457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2236,12 +1658,12 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Unquenched lifetime: the longest of the usable measurements, because residual oxygen can only shorten it.</t>
+          <t>Unquenched lifetime, single-exponential fit of pc_tcspc/PC&lt;n&gt;.txt.</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>experimental_data_raw/pc_tcspc/lifetimes_tau0.csv: tau0_ns</t>
+          <t>experimental_data_raw/pc_tcspc/lifetimes_tcspc.csv: tau0_ns</t>
         </is>
       </c>
     </row>
@@ -2253,7 +1675,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>tau0_std / ns</t>
+          <t>tau0_err / ns</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
@@ -2263,12 +1685,12 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Spread across repeats; with one measurement, that fit's standard error.</t>
+          <t>Standard error of that fit.</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>experimental_data_raw/pc_tcspc/lifetimes_tau0.csv: tau0_std_ns</t>
+          <t>experimental_data_raw/pc_tcspc/lifetimes_tcspc.csv: tau0_err_ns</t>
         </is>
       </c>
     </row>
@@ -2280,186 +1702,71 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>tau0_rsd</t>
+          <t>tau0_note</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr"/>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>tau0_std / tau0.</t>
+          <t>Deviation from the standard fit window.</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>experimental_data_raw/pc_tcspc/lifetimes_tau0.csv: tau0_rsd</t>
+          <t>experimental_data_raw/pc_tcspc/lifetimes_tcspc.csv: note</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Excited-state lifetime, TCSPC in MeCN under Ar</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>n_measurements</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr"/>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Usable traces behind tau0.</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>experimental_data_raw/pc_tcspc/lifetimes_tau0.csv: n_measurements</t>
-        </is>
-      </c>
+      <c r="A11" s="12" t="n"/>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="13" t="n"/>
+      <c r="E11" s="12" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>Excited-state lifetime, TCSPC in MeCN under Ar</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>n_traces_rejected</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr"/>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Traces dropped as duplicates, unfitted, or with too short a window.</t>
-        </is>
-      </c>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>experimental_data_raw/pc_tcspc/lifetimes_tau0.csv: n_traces_rejected</t>
-        </is>
-      </c>
+          <t>One row per photocatalyst with a compound record. PC7 and PC26 are not in the screen</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="12" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>Excited-state lifetime, TCSPC in MeCN under Ar</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>tau0_consistent</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr"/>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>With repeats: 1 if they agree within 10 %, 0 if not. Blank for one measurement.</t>
-        </is>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>experimental_data_raw/pc_tcspc/lifetimes_tau0.csv: consistent</t>
-        </is>
-      </c>
+          <t>and have no lifetime. PC24 is in the screen and excluded from the dataset in</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="12" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>Excited-state lifetime, TCSPC in MeCN under Ar</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>trace_used</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr"/>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>The trace tau0 is taken from.</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>experimental_data_raw/pc_tcspc/lifetimes_tau0.csv: trace_used</t>
-        </is>
-      </c>
+          <t>dataset/build_dataset.py, not here.</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="12" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>Excited-state lifetime, TCSPC in MeCN under Ar</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>tau0_note</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr"/>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>How tau0 was selected, and what was rejected.</t>
-        </is>
-      </c>
-      <c r="E15" s="12" t="inlineStr">
-        <is>
-          <t>experimental_data_raw/pc_tcspc/lifetimes_tau0.csv: note</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="12" t="n"/>
-      <c r="D16" s="13" t="n"/>
-      <c r="E16" s="12" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>One row per photocatalyst with a compound record. PC7 was measured but is not in the</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="n"/>
-      <c r="C17" s="12" t="n"/>
-      <c r="D17" s="13" t="n"/>
-      <c r="E17" s="12" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>screen; PC26 has no record beyond its number. PC24 is in the screen and excluded from</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="13" t="n"/>
-      <c r="E18" s="12" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>the dataset in dataset/build_dataset.py, not here.</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="13" t="n"/>
-      <c r="E19" s="12" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
           <t>Read with pandas as: pd.read_excel(path, header=1), then drop the 'Unnamed' columns.</t>
         </is>
       </c>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="13" t="n"/>
-      <c r="E20" s="12" t="n"/>
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="12" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>